<commit_message>
More Changes. Happy with the current state of the package, thus the commit
</commit_message>
<xml_diff>
--- a/data/example_data.xlsx
+++ b/data/example_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\david\R_Projects\xafty\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DE151AF-0051-4321-86AD-808F0E38264D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{354439E4-0F50-4500-9965-19B873EF7BBE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{8DFAE3C1-B59B-48F9-BE9F-315C3CF6D3D2}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="20">
   <si>
     <t>Name</t>
   </si>
@@ -53,18 +53,6 @@
     <t>no</t>
   </si>
   <si>
-    <t>David</t>
-  </si>
-  <si>
-    <t>Diana</t>
-  </si>
-  <si>
-    <t>Lena</t>
-  </si>
-  <si>
-    <t>Marcel</t>
-  </si>
-  <si>
     <t>Mail</t>
   </si>
   <si>
@@ -77,16 +65,37 @@
     <t>Lena_pompena_420@gmail.com</t>
   </si>
   <si>
+    <t>Date_2</t>
+  </si>
+  <si>
+    <t>Date_3</t>
+  </si>
+  <si>
+    <t>01.01.1998</t>
+  </si>
+  <si>
+    <t>Davidb</t>
+  </si>
+  <si>
+    <t>Dianab</t>
+  </si>
+  <si>
+    <t>Lenab</t>
+  </si>
+  <si>
+    <t>Marcelb</t>
+  </si>
+  <si>
     <t>Marcel_crone@doodle.com</t>
   </si>
   <si>
-    <t>Date_2</t>
-  </si>
-  <si>
-    <t>Date_3</t>
-  </si>
-  <si>
-    <t>01.01.1998</t>
+    <t>01.01.1999</t>
+  </si>
+  <si>
+    <t>01.01.2000</t>
+  </si>
+  <si>
+    <t>01.01.2001</t>
   </si>
 </sst>
 </file>
@@ -96,7 +105,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-809]dd\ mmmm\ yyyy;@"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -108,6 +117,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -480,18 +495,18 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" t="s">
         <v>9</v>
       </c>
-      <c r="F1" t="s">
-        <v>14</v>
-      </c>
       <c r="G1" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="B2" s="3">
         <v>34184</v>
@@ -503,18 +518,18 @@
         <v>4</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F2" s="5">
         <v>36750</v>
       </c>
       <c r="G2" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="B3" s="3">
         <v>36665</v>
@@ -526,12 +541,18 @@
         <v>4</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
+      </c>
+      <c r="F3" s="5">
+        <v>36751</v>
+      </c>
+      <c r="G3" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="B4" s="3">
         <v>37904</v>
@@ -543,12 +564,18 @@
         <v>4</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>12</v>
+        <v>8</v>
+      </c>
+      <c r="F4" s="5">
+        <v>36752</v>
+      </c>
+      <c r="G4" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B5" s="3">
         <v>34955</v>
@@ -560,10 +587,17 @@
         <v>4</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>13</v>
+        <v>16</v>
+      </c>
+      <c r="F5" s="5">
+        <v>36753</v>
+      </c>
+      <c r="G5" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1" xr:uid="{B97C25F1-0918-49BE-9BB7-885BD3F2EE68}"/>
     <hyperlink ref="E3" r:id="rId2" xr:uid="{F61677AF-28A4-44C4-BAE6-B73DA6A27213}"/>

</xml_diff>